<commit_message>
Complete Day 37 cluster profiling and statistics
</commit_message>
<xml_diff>
--- a/output/cluster_results.xlsx
+++ b/output/cluster_results.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>High Risk</t>
+          <t>Turnaround</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3459,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4242,7 +4242,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>High Risk</t>
+          <t>Turnaround</t>
         </is>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5725,7 +5725,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6020,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6390,7 +6390,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6685,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>High Quality</t>
         </is>
       </c>
     </row>

</xml_diff>